<commit_message>
bind final q2412 attachments and review
</commit_message>
<xml_diff>
--- a/task/关键标准答案.xlsx
+++ b/task/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R827a952f583f421a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R331d3f38169948f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R45064d63010d4df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Reee97f9330864959"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Rfb8b0067a3dd430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="Rdb35da963e9443bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Ra924d28c639c4282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R0042d3adf69d48e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R3adad1d1ab5247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Rb66617464e1045dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -313,13 +313,13 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>阶段清单</x:v>
+        <x:v>steady阶段清单</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>output/rendered/阶段名.yaml</x:v>
+        <x:v>output/rendered/steady.yaml</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>供发布评审核对对象和引用</x:v>
+        <x:v>供发布评审核对旧钥稳定状态</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
         <x:v>按phase主键解析YAML</x:v>
@@ -327,57 +327,99 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>轮换台账</x:v>
+        <x:v>preload阶段清单</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>output/reports/rotation_ledger.csv</x:v>
+        <x:v>output/rendered/preload.yaml</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
-        <x:v>连接阶段计划与清单</x:v>
+        <x:v>供发布评审核对新钥预载</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
-        <x:v>按phase逐字段核对</x:v>
+        <x:v>按phase主键解析YAML</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="5" t="str">
-        <x:v>Secret引用核对</x:v>
+        <x:v>activate阶段清单</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>output/reports/secret_reference_review.csv</x:v>
+        <x:v>output/rendered/activate.yaml</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>连接Secret登记与投影源</x:v>
+        <x:v>供发布评审核对新钥启用</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>按phase和projection_order核对</x:v>
+        <x:v>按phase主键解析YAML</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="5" t="str">
+        <x:v>retire阶段清单</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="str">
+        <x:v>output/rendered/retire.yaml</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="str">
+        <x:v>供发布评审核对旧钥退场</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="str">
+        <x:v>按phase主键解析YAML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="5" t="str">
+        <x:v>轮换台账</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="str">
+        <x:v>output/reports/rotation_ledger.csv</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="str">
+        <x:v>连接阶段计划与清单</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>按phase逐字段核对</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="5" t="str">
+        <x:v>Secret引用核对</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>output/reports/secret_reference_review.csv</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="str">
+        <x:v>连接Secret登记与投影源</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>按phase和projection_order核对</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="5" t="str">
         <x:v>变更说明</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B9" s="5" t="str">
         <x:v>output/change_note.md</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C9" s="5" t="str">
         <x:v>说明维护窗、顺序、回滚与分工</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D9" s="5" t="str">
         <x:v>与change_request.md比较</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="6" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
         <x:v>使用说明</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="str">
+      <x:c r="B10" s="6" t="str">
         <x:v>output/README.md</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="str">
+      <x:c r="C10" s="6" t="str">
         <x:v>说明目录用途</x:v>
       </x:c>
-      <x:c r="D7" s="6" t="str">
+      <x:c r="D10" s="6" t="str">
         <x:v>核对实际路径</x:v>
       </x:c>
     </x:row>

</xml_diff>